<commit_message>
Atualização automática convênios de entrada
</commit_message>
<xml_diff>
--- a/link_convenios.xlsx
+++ b/link_convenios.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$B$1338</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="916">
   <si>
     <t>https://drive.google.com/file/d/1mnH14gEK5_xghzIJ-rHHZ8lOxqCsVnB8/view</t>
   </si>
@@ -2128,9 +2128,6 @@
     <t>https://portaldatransparencia.gov.br/emendas/detalhe?codigoEmenda=202040160001</t>
   </si>
   <si>
-    <t xml:space="preserve"> https://portaldatransparencia.gov.br/emendas/detalhe?codigoEmenda=202040640005</t>
-  </si>
-  <si>
     <t>https://portaldatransparencia.gov.br/emendas/detalhe?codigoEmenda=202041570012</t>
   </si>
   <si>
@@ -2759,13 +2756,46 @@
   </si>
   <si>
     <t>https://nuvem.cge.mg.gov.br/index.php/s/QGEF6HJfKz55skW</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/nHXkEAn4WjkeoWk</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/9g3q5eMfzEFyj23</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/J99nADnJKCcnGjJ</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/YfrtYwPF9RC27D4</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/rTWFSQkkcD7Q4Z3</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/G5gqNmAmJBG3ibE</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/wW6y7eQ9ZkSAyRC</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/pdHbaWxErwL7ziB</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/YFXL6dS4HfF3ZTE</t>
+  </si>
+  <si>
+    <t>https://portaldatransparencia.gov.br/emendas/detalhe?codigoEmenda=202643430001&amp;codigoTipoEmenda=1&amp;ordenarPor=codigoEmpenhoResumido&amp;direcao=desc</t>
+  </si>
+  <si>
+    <t>https://portaldatransparencia.gov.br/emendas/detalhe?codigoEmenda=202638970005&amp;codigoTipoEmenda=1&amp;ordenarPor=codigoEmpenhoResumido&amp;direcao=asc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2777,6 +2807,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2811,16 +2849,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3158,10 +3199,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15">
       <c r="A1" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -3169,7 +3210,7 @@
         <v>9270124</v>
       </c>
       <c r="B2" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -3177,7 +3218,7 @@
         <v>9270144</v>
       </c>
       <c r="B3" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -3185,7 +3226,7 @@
         <v>9270149</v>
       </c>
       <c r="B4" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -3193,7 +3234,7 @@
         <v>9270192</v>
       </c>
       <c r="B5" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -3201,7 +3242,7 @@
         <v>9270199</v>
       </c>
       <c r="B6" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -3209,7 +3250,7 @@
         <v>9270223</v>
       </c>
       <c r="B7" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -3217,7 +3258,7 @@
         <v>9270245</v>
       </c>
       <c r="B8" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -3225,7 +3266,7 @@
         <v>9270257</v>
       </c>
       <c r="B9" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -3238,7 +3279,7 @@
         <v>9270802</v>
       </c>
       <c r="B11" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -3246,7 +3287,7 @@
         <v>9270942</v>
       </c>
       <c r="B12" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -3254,7 +3295,7 @@
         <v>9270958</v>
       </c>
       <c r="B13" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -3262,7 +3303,7 @@
         <v>9271592</v>
       </c>
       <c r="B14" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -3270,7 +3311,7 @@
         <v>9271602</v>
       </c>
       <c r="B15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -3278,7 +3319,7 @@
         <v>9271647</v>
       </c>
       <c r="B16" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -3336,7 +3377,7 @@
         <v>9274488</v>
       </c>
       <c r="B27" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -3344,7 +3385,7 @@
         <v>9274495</v>
       </c>
       <c r="B28" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -3352,7 +3393,7 @@
         <v>9274497</v>
       </c>
       <c r="B29" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -3365,7 +3406,7 @@
         <v>9275416</v>
       </c>
       <c r="B31" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -3398,7 +3439,7 @@
         <v>9276559</v>
       </c>
       <c r="B37" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -3411,7 +3452,7 @@
         <v>9276562</v>
       </c>
       <c r="B39" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -3419,7 +3460,7 @@
         <v>9276568</v>
       </c>
       <c r="B40" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -3432,7 +3473,7 @@
         <v>9277512</v>
       </c>
       <c r="B42" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -3445,7 +3486,7 @@
         <v>9279529</v>
       </c>
       <c r="B44" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -3453,7 +3494,7 @@
         <v>9280371</v>
       </c>
       <c r="B45" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -3461,7 +3502,7 @@
         <v>9280479</v>
       </c>
       <c r="B46" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -3509,7 +3550,7 @@
         <v>9282915</v>
       </c>
       <c r="B55" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -3517,7 +3558,7 @@
         <v>9282916</v>
       </c>
       <c r="B56" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -3525,7 +3566,7 @@
         <v>9282958</v>
       </c>
       <c r="B57" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -3533,7 +3574,7 @@
         <v>9283109</v>
       </c>
       <c r="B58" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -3556,7 +3597,7 @@
         <v>9285205</v>
       </c>
       <c r="B62" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -3574,7 +3615,7 @@
         <v>9286434</v>
       </c>
       <c r="B65" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -3597,7 +3638,7 @@
         <v>9288048</v>
       </c>
       <c r="B69" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -3778,7 +3819,7 @@
         <v>9288155</v>
       </c>
       <c r="B92" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -4026,7 +4067,7 @@
         <v>9288250</v>
       </c>
       <c r="B123" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="124" spans="1:2">
@@ -4034,7 +4075,7 @@
         <v>9288331</v>
       </c>
       <c r="B124" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="125" spans="1:2">
@@ -4042,7 +4083,7 @@
         <v>9288332</v>
       </c>
       <c r="B125" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="126" spans="1:2">
@@ -4218,7 +4259,7 @@
         <v>9288360</v>
       </c>
       <c r="B147" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="148" spans="1:2">
@@ -4226,15 +4267,15 @@
         <v>9288361</v>
       </c>
       <c r="B148" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149">
         <v>9288362</v>
       </c>
-      <c r="B149" t="s">
-        <v>695</v>
+      <c r="B149" s="2" t="s">
+        <v>697</v>
       </c>
     </row>
     <row r="150" spans="1:2">
@@ -4250,15 +4291,15 @@
         <v>9288369</v>
       </c>
       <c r="B151" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="152" spans="1:2">
       <c r="A152">
         <v>9288370</v>
       </c>
-      <c r="B152" t="s">
-        <v>695</v>
+      <c r="B152" s="2" t="s">
+        <v>697</v>
       </c>
     </row>
     <row r="153" spans="1:2">
@@ -4289,8 +4330,8 @@
       <c r="A156">
         <v>9289863</v>
       </c>
-      <c r="B156" t="s">
-        <v>695</v>
+      <c r="B156" s="2" t="s">
+        <v>697</v>
       </c>
     </row>
     <row r="157" spans="1:2">
@@ -4372,7 +4413,7 @@
         <v>9291962</v>
       </c>
       <c r="B167" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="168" spans="1:2">
@@ -4380,7 +4421,7 @@
         <v>9291964</v>
       </c>
       <c r="B168" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="169" spans="1:2">
@@ -4388,7 +4429,7 @@
         <v>9291965</v>
       </c>
       <c r="B169" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="170" spans="1:2">
@@ -4396,7 +4437,7 @@
         <v>9291966</v>
       </c>
       <c r="B170" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="171" spans="1:2">
@@ -4404,7 +4445,7 @@
         <v>9291967</v>
       </c>
       <c r="B171" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="172" spans="1:2">
@@ -4433,7 +4474,7 @@
         <v>9292038</v>
       </c>
       <c r="B175" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="176" spans="1:2">
@@ -4553,7 +4594,7 @@
         <v>9293668</v>
       </c>
       <c r="B193" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="194" spans="1:2">
@@ -4590,7 +4631,7 @@
         <v>9294158</v>
       </c>
       <c r="B198" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
     <row r="199" spans="1:2">
@@ -4622,7 +4663,7 @@
         <v>9301342</v>
       </c>
       <c r="B202" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="203" spans="1:2">
@@ -4630,7 +4671,7 @@
         <v>9301344</v>
       </c>
       <c r="B203" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="204" spans="1:2">
@@ -4744,7 +4785,7 @@
         <v>9313095</v>
       </c>
       <c r="B218" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="219" spans="1:2">
@@ -4778,7 +4819,7 @@
         <v>9314782</v>
       </c>
       <c r="B223" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="224" spans="1:2">
@@ -4791,7 +4832,7 @@
         <v>9315157</v>
       </c>
       <c r="B225" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="226" spans="1:2">
@@ -4799,7 +4840,7 @@
         <v>9315170</v>
       </c>
       <c r="B226" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="227" spans="1:2">
@@ -4833,7 +4874,7 @@
         <v>9315350</v>
       </c>
       <c r="B231" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="232" spans="1:2">
@@ -4846,7 +4887,7 @@
         <v>9315513</v>
       </c>
       <c r="B233" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="234" spans="1:2">
@@ -4887,11 +4928,17 @@
       <c r="A239">
         <v>9317170</v>
       </c>
+      <c r="B239" t="s">
+        <v>913</v>
+      </c>
     </row>
     <row r="240" spans="1:2">
       <c r="A240">
         <v>9317172</v>
       </c>
+      <c r="B240" t="s">
+        <v>908</v>
+      </c>
     </row>
     <row r="241" spans="1:2">
       <c r="A241">
@@ -4948,7 +4995,7 @@
         <v>9317481</v>
       </c>
       <c r="B248" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="249" spans="1:2">
@@ -4956,7 +5003,7 @@
         <v>9317482</v>
       </c>
       <c r="B249" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="250" spans="1:2">
@@ -5040,7 +5087,7 @@
         <v>9318434</v>
       </c>
       <c r="B264" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="265" spans="1:2">
@@ -5048,7 +5095,7 @@
         <v>9318436</v>
       </c>
       <c r="B265" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="266" spans="1:2">
@@ -5056,7 +5103,7 @@
         <v>9318486</v>
       </c>
       <c r="B266" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="267" spans="1:2">
@@ -5064,7 +5111,7 @@
         <v>9318699</v>
       </c>
       <c r="B267" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="268" spans="1:2">
@@ -5093,7 +5140,7 @@
         <v>9318764</v>
       </c>
       <c r="B271" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="272" spans="1:2">
@@ -5130,6 +5177,9 @@
       <c r="A278">
         <v>9319167</v>
       </c>
+      <c r="B278" t="s">
+        <v>909</v>
+      </c>
     </row>
     <row r="279" spans="1:2">
       <c r="A279">
@@ -5141,7 +5191,7 @@
         <v>9319190</v>
       </c>
       <c r="B280" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="281" spans="1:2">
@@ -5157,7 +5207,7 @@
         <v>9319193</v>
       </c>
       <c r="B282" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="283" spans="1:2">
@@ -5170,7 +5220,7 @@
         <v>9319206</v>
       </c>
       <c r="B284" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="285" spans="1:2">
@@ -5178,7 +5228,7 @@
         <v>9319209</v>
       </c>
       <c r="B285" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="286" spans="1:2">
@@ -5186,7 +5236,7 @@
         <v>9319210</v>
       </c>
       <c r="B286" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="287" spans="1:2">
@@ -5194,7 +5244,7 @@
         <v>9319211</v>
       </c>
       <c r="B287" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="288" spans="1:2">
@@ -5207,7 +5257,7 @@
         <v>9319439</v>
       </c>
       <c r="B289" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="290" spans="1:2">
@@ -5215,7 +5265,7 @@
         <v>9320345</v>
       </c>
       <c r="B290" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="291" spans="1:2">
@@ -5223,7 +5273,7 @@
         <v>9321167</v>
       </c>
       <c r="B291" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="292" spans="1:2">
@@ -5231,7 +5281,7 @@
         <v>9321196</v>
       </c>
       <c r="B292" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
     </row>
     <row r="293" spans="1:2">
@@ -5239,7 +5289,7 @@
         <v>9321263</v>
       </c>
       <c r="B293" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="294" spans="1:2">
@@ -5255,7 +5305,7 @@
         <v>9321271</v>
       </c>
       <c r="B295" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="296" spans="1:2">
@@ -5273,7 +5323,7 @@
         <v>9322361</v>
       </c>
       <c r="B298" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="299" spans="1:2">
@@ -5331,7 +5381,7 @@
         <v>9323348</v>
       </c>
       <c r="B309" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="310" spans="1:2">
@@ -5344,7 +5394,7 @@
         <v>9324016</v>
       </c>
       <c r="B311" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
     </row>
     <row r="312" spans="1:2">
@@ -5360,7 +5410,7 @@
         <v>9324182</v>
       </c>
       <c r="B313" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
     </row>
     <row r="314" spans="1:2">
@@ -5381,7 +5431,7 @@
         <v>9324187</v>
       </c>
       <c r="B316" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="317" spans="1:2">
@@ -5389,7 +5439,7 @@
         <v>9324188</v>
       </c>
       <c r="B317" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="318" spans="1:2">
@@ -5397,7 +5447,7 @@
         <v>9324189</v>
       </c>
       <c r="B318" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="319" spans="1:2">
@@ -5405,7 +5455,7 @@
         <v>9324191</v>
       </c>
       <c r="B319" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="320" spans="1:2">
@@ -5418,7 +5468,7 @@
         <v>9325274</v>
       </c>
       <c r="B321" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="322" spans="1:2">
@@ -5439,7 +5489,7 @@
         <v>9325286</v>
       </c>
       <c r="B324" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="325" spans="1:2">
@@ -5447,7 +5497,7 @@
         <v>9325287</v>
       </c>
       <c r="B325" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="326" spans="1:2">
@@ -5455,7 +5505,7 @@
         <v>9325288</v>
       </c>
       <c r="B326" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="327" spans="1:2">
@@ -5498,7 +5548,7 @@
         <v>9327216</v>
       </c>
       <c r="B334" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="335" spans="1:2">
@@ -5808,7 +5858,7 @@
         <v>9340452</v>
       </c>
       <c r="B384" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
     </row>
     <row r="385" spans="1:2">
@@ -5834,7 +5884,7 @@
         <v>9340589</v>
       </c>
       <c r="B388" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="389" spans="1:2">
@@ -5871,7 +5921,7 @@
         <v>9341289</v>
       </c>
       <c r="B393" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="394" spans="1:2">
@@ -5907,7 +5957,7 @@
         <v>9341516</v>
       </c>
       <c r="B399" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="400" spans="1:2">
@@ -5969,7 +6019,7 @@
         <v>9342915</v>
       </c>
       <c r="B409" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="410" spans="1:2">
@@ -6013,7 +6063,7 @@
         <v>9344036</v>
       </c>
       <c r="B416" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="417" spans="1:2">
@@ -6050,7 +6100,7 @@
         <v>9344115</v>
       </c>
       <c r="B421" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="422" spans="1:2">
@@ -6066,7 +6116,7 @@
         <v>9344189</v>
       </c>
       <c r="B423" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="424" spans="1:2">
@@ -6074,7 +6124,7 @@
         <v>9344197</v>
       </c>
       <c r="B424" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="425" spans="1:2">
@@ -6082,7 +6132,7 @@
         <v>9344199</v>
       </c>
       <c r="B425" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="426" spans="1:2">
@@ -6121,7 +6171,7 @@
         <v>9344645</v>
       </c>
       <c r="B431" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="432" spans="1:2">
@@ -6174,7 +6224,7 @@
         <v>9344844</v>
       </c>
       <c r="B438" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="439" spans="1:2">
@@ -6280,7 +6330,7 @@
         <v>9345607</v>
       </c>
       <c r="B452" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="453" spans="1:2">
@@ -6303,7 +6353,7 @@
         <v>9345820</v>
       </c>
       <c r="B456" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="457" spans="1:2">
@@ -6390,7 +6440,7 @@
         <v>9346153</v>
       </c>
       <c r="B471" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="472" spans="1:2">
@@ -6398,7 +6448,7 @@
         <v>9346288</v>
       </c>
       <c r="B472" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="473" spans="1:2">
@@ -6478,7 +6528,7 @@
         <v>9348878</v>
       </c>
       <c r="B485" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
     </row>
     <row r="486" spans="1:2">
@@ -6486,7 +6536,7 @@
         <v>9349512</v>
       </c>
       <c r="B486" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="487" spans="1:2">
@@ -6507,7 +6557,7 @@
         <v>9349516</v>
       </c>
       <c r="B489" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="490" spans="1:2">
@@ -6515,7 +6565,7 @@
         <v>9350464</v>
       </c>
       <c r="B490" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
     </row>
     <row r="491" spans="1:2">
@@ -6539,7 +6589,7 @@
         <v>9359872</v>
       </c>
       <c r="B493" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="494" spans="1:2">
@@ -6560,7 +6610,7 @@
         <v>9361850</v>
       </c>
       <c r="B496" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="497" spans="1:2">
@@ -6586,7 +6636,7 @@
         <v>9362450</v>
       </c>
       <c r="B500" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="501" spans="1:2">
@@ -6599,7 +6649,7 @@
         <v>9363607</v>
       </c>
       <c r="B502" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="503" spans="1:2">
@@ -6607,7 +6657,7 @@
         <v>9363624</v>
       </c>
       <c r="B503" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="504" spans="1:2">
@@ -6625,7 +6675,7 @@
         <v>9368834</v>
       </c>
       <c r="B506" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="507" spans="1:2">
@@ -6718,7 +6768,7 @@
         <v>9370613</v>
       </c>
       <c r="B518" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="519" spans="1:2">
@@ -6731,7 +6781,7 @@
         <v>9370628</v>
       </c>
       <c r="B520" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="521" spans="1:2">
@@ -6739,7 +6789,7 @@
         <v>9370631</v>
       </c>
       <c r="B521" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="522" spans="1:2">
@@ -6842,7 +6892,7 @@
         <v>9372113</v>
       </c>
       <c r="B538" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="539" spans="1:2">
@@ -6850,7 +6900,7 @@
         <v>9372385</v>
       </c>
       <c r="B539" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="540" spans="1:2">
@@ -6863,7 +6913,7 @@
         <v>9372558</v>
       </c>
       <c r="B541" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
     </row>
     <row r="542" spans="1:2">
@@ -6884,7 +6934,7 @@
         <v>9372564</v>
       </c>
       <c r="B544" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="545" spans="1:2">
@@ -6907,7 +6957,7 @@
         <v>9372625</v>
       </c>
       <c r="B548" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
     </row>
     <row r="549" spans="1:2">
@@ -6915,7 +6965,7 @@
         <v>9372627</v>
       </c>
       <c r="B549" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
     </row>
     <row r="550" spans="1:2">
@@ -6928,7 +6978,7 @@
         <v>9372706</v>
       </c>
       <c r="B551" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="552" spans="1:2">
@@ -6946,7 +6996,7 @@
         <v>9372843</v>
       </c>
       <c r="B554" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
     </row>
     <row r="555" spans="1:2">
@@ -6967,7 +7017,7 @@
         <v>9376674</v>
       </c>
       <c r="B557" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="558" spans="1:2">
@@ -7039,6 +7089,9 @@
       <c r="A568">
         <v>9386240</v>
       </c>
+      <c r="B568" t="s">
+        <v>905</v>
+      </c>
     </row>
     <row r="569" spans="1:2">
       <c r="A569">
@@ -7068,7 +7121,7 @@
         <v>9388834</v>
       </c>
       <c r="B573" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="574" spans="1:2">
@@ -7085,6 +7138,9 @@
       <c r="A576">
         <v>9389062</v>
       </c>
+      <c r="B576" t="s">
+        <v>906</v>
+      </c>
     </row>
     <row r="577" spans="1:2">
       <c r="A577">
@@ -7296,7 +7352,7 @@
         <v>9390538</v>
       </c>
       <c r="B603" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="604" spans="1:2">
@@ -7360,7 +7416,7 @@
         <v>9392826</v>
       </c>
       <c r="B611" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="612" spans="1:2">
@@ -7408,7 +7464,7 @@
         <v>9393466</v>
       </c>
       <c r="B617" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
     </row>
     <row r="618" spans="1:2">
@@ -7527,13 +7583,16 @@
       <c r="A632">
         <v>9396780</v>
       </c>
+      <c r="B632" t="s">
+        <v>907</v>
+      </c>
     </row>
     <row r="633" spans="1:2">
       <c r="A633">
         <v>9397802</v>
       </c>
       <c r="B633" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="634" spans="1:2">
@@ -7610,7 +7669,7 @@
         <v>9401387</v>
       </c>
       <c r="B643" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="644" spans="1:2">
@@ -7618,7 +7677,7 @@
         <v>9401388</v>
       </c>
       <c r="B644" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="645" spans="1:2">
@@ -7691,7 +7750,7 @@
         <v>9404003</v>
       </c>
       <c r="B655" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="656" spans="1:2">
@@ -7699,7 +7758,7 @@
         <v>9404005</v>
       </c>
       <c r="B656" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="657" spans="1:2">
@@ -8135,7 +8194,7 @@
         <v>9408775</v>
       </c>
       <c r="B715" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="716" spans="1:2">
@@ -8285,7 +8344,7 @@
         <v>9409727</v>
       </c>
       <c r="B736" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
     </row>
     <row r="737" spans="1:2">
@@ -8301,7 +8360,7 @@
         <v>9409731</v>
       </c>
       <c r="B738" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="739" spans="1:2">
@@ -8322,7 +8381,7 @@
         <v>9409756</v>
       </c>
       <c r="B741" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="742" spans="1:2">
@@ -8338,7 +8397,7 @@
         <v>9410094</v>
       </c>
       <c r="B743" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
     </row>
     <row r="744" spans="1:2">
@@ -8919,16 +8978,25 @@
       <c r="A821">
         <v>9433735</v>
       </c>
+      <c r="B821" t="s">
+        <v>911</v>
+      </c>
     </row>
     <row r="822" spans="1:2">
       <c r="A822">
         <v>9433736</v>
       </c>
+      <c r="B822" t="s">
+        <v>912</v>
+      </c>
     </row>
     <row r="823" spans="1:2">
       <c r="A823">
         <v>9433738</v>
       </c>
+      <c r="B823" t="s">
+        <v>910</v>
+      </c>
     </row>
     <row r="824" spans="1:2">
       <c r="A824">
@@ -9433,7 +9501,7 @@
         <v>9445638</v>
       </c>
       <c r="B887" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="888" spans="1:2">
@@ -9465,7 +9533,7 @@
         <v>9445646</v>
       </c>
       <c r="B891" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="892" spans="1:2">
@@ -9577,7 +9645,7 @@
         <v>9445733</v>
       </c>
       <c r="B905" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="906" spans="1:2">
@@ -9593,7 +9661,7 @@
         <v>9445735</v>
       </c>
       <c r="B907" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="908" spans="1:2">
@@ -9601,7 +9669,7 @@
         <v>9445736</v>
       </c>
       <c r="B908" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="909" spans="1:2">
@@ -9609,7 +9677,7 @@
         <v>9445737</v>
       </c>
       <c r="B909" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="910" spans="1:2">
@@ -9617,7 +9685,7 @@
         <v>9445738</v>
       </c>
       <c r="B910" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="911" spans="1:2">
@@ -9625,7 +9693,7 @@
         <v>9445739</v>
       </c>
       <c r="B911" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="912" spans="1:2">
@@ -9849,7 +9917,7 @@
         <v>9447476</v>
       </c>
       <c r="B939" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="940" spans="1:2">
@@ -9881,7 +9949,7 @@
         <v>9447499</v>
       </c>
       <c r="B943" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="944" spans="1:2">
@@ -9889,7 +9957,7 @@
         <v>9447502</v>
       </c>
       <c r="B944" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="945" spans="1:2">
@@ -9905,7 +9973,7 @@
         <v>9447747</v>
       </c>
       <c r="B946" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="947" spans="1:2">
@@ -9993,7 +10061,7 @@
         <v>9447779</v>
       </c>
       <c r="B957" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="958" spans="1:2">
@@ -10017,7 +10085,7 @@
         <v>9447803</v>
       </c>
       <c r="B960" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="961" spans="1:2">
@@ -10025,7 +10093,7 @@
         <v>9447912</v>
       </c>
       <c r="B961" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="962" spans="1:2">
@@ -10033,7 +10101,7 @@
         <v>9450222</v>
       </c>
       <c r="B962" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="963" spans="1:2">
@@ -10049,7 +10117,7 @@
         <v>9451351</v>
       </c>
       <c r="B964" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="965" spans="1:2">
@@ -10105,7 +10173,7 @@
         <v>9453523</v>
       </c>
       <c r="B971" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="972" spans="1:2">
@@ -10498,7 +10566,7 @@
         <v>9461430</v>
       </c>
       <c r="B1022" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="1023" spans="1:2">
@@ -10511,7 +10579,7 @@
         <v>9461432</v>
       </c>
       <c r="B1024" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="1025" spans="1:2">
@@ -10534,7 +10602,7 @@
         <v>9461437</v>
       </c>
       <c r="B1028" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="1029" spans="1:2">
@@ -10542,7 +10610,7 @@
         <v>9461439</v>
       </c>
       <c r="B1029" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="1030" spans="1:2">
@@ -10550,7 +10618,7 @@
         <v>9461440</v>
       </c>
       <c r="B1030" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="1031" spans="1:2">
@@ -10558,7 +10626,7 @@
         <v>9461441</v>
       </c>
       <c r="B1031" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
     </row>
     <row r="1032" spans="1:2">
@@ -10566,7 +10634,7 @@
         <v>9461443</v>
       </c>
       <c r="B1032" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="1033" spans="1:2">
@@ -10574,7 +10642,7 @@
         <v>9461445</v>
       </c>
       <c r="B1033" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
     </row>
     <row r="1034" spans="1:2">
@@ -10582,7 +10650,7 @@
         <v>9461446</v>
       </c>
       <c r="B1034" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="1035" spans="1:2">
@@ -10590,7 +10658,7 @@
         <v>9461447</v>
       </c>
       <c r="B1035" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="1036" spans="1:2">
@@ -10598,7 +10666,7 @@
         <v>9461449</v>
       </c>
       <c r="B1036" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="1037" spans="1:2">
@@ -10606,7 +10674,7 @@
         <v>9461451</v>
       </c>
       <c r="B1037" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="1038" spans="1:2">
@@ -10614,7 +10682,7 @@
         <v>9461453</v>
       </c>
       <c r="B1038" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="1039" spans="1:2">
@@ -10622,7 +10690,7 @@
         <v>9461454</v>
       </c>
       <c r="B1039" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
     </row>
     <row r="1040" spans="1:2">
@@ -10630,7 +10698,7 @@
         <v>9461456</v>
       </c>
       <c r="B1040" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="1041" spans="1:2">
@@ -10638,7 +10706,7 @@
         <v>9461458</v>
       </c>
       <c r="B1041" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
     </row>
     <row r="1042" spans="1:2">
@@ -10654,7 +10722,7 @@
         <v>9461460</v>
       </c>
       <c r="B1043" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
     </row>
     <row r="1044" spans="1:2">
@@ -10662,7 +10730,7 @@
         <v>9461461</v>
       </c>
       <c r="B1044" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
     </row>
     <row r="1045" spans="1:2">
@@ -10670,7 +10738,7 @@
         <v>9461462</v>
       </c>
       <c r="B1045" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="1046" spans="1:2">
@@ -10678,7 +10746,7 @@
         <v>9461463</v>
       </c>
       <c r="B1046" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="1047" spans="1:2">
@@ -10686,7 +10754,7 @@
         <v>9468050</v>
       </c>
       <c r="B1047" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
     <row r="1048" spans="1:2">
@@ -10702,7 +10770,7 @@
         <v>9468052</v>
       </c>
       <c r="B1049" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="1050" spans="1:2">
@@ -10734,7 +10802,7 @@
         <v>9468059</v>
       </c>
       <c r="B1053" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="1054" spans="1:2">
@@ -10742,7 +10810,7 @@
         <v>9468061</v>
       </c>
       <c r="B1054" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
     </row>
     <row r="1055" spans="1:2">
@@ -10750,7 +10818,7 @@
         <v>9468062</v>
       </c>
       <c r="B1055" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
     </row>
     <row r="1056" spans="1:2">
@@ -10774,7 +10842,7 @@
         <v>9468435</v>
       </c>
       <c r="B1058" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="1059" spans="1:2">
@@ -10870,7 +10938,7 @@
         <v>9470477</v>
       </c>
       <c r="B1070" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="1071" spans="1:2">
@@ -10878,7 +10946,7 @@
         <v>9470534</v>
       </c>
       <c r="B1071" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="1072" spans="1:2">
@@ -10886,7 +10954,7 @@
         <v>9470535</v>
       </c>
       <c r="B1072" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="1073" spans="1:2">
@@ -10894,7 +10962,7 @@
         <v>9470539</v>
       </c>
       <c r="B1073" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="1074" spans="1:2">
@@ -10910,7 +10978,7 @@
         <v>9470656</v>
       </c>
       <c r="B1075" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="1076" spans="1:2">
@@ -10926,7 +10994,7 @@
         <v>9471205</v>
       </c>
       <c r="B1077" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="1078" spans="1:2">
@@ -10990,7 +11058,7 @@
         <v>9473170</v>
       </c>
       <c r="B1085" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="1086" spans="1:2">
@@ -10998,7 +11066,7 @@
         <v>9473171</v>
       </c>
       <c r="B1086" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="1087" spans="1:2">
@@ -11371,7 +11439,7 @@
         <v>9479195</v>
       </c>
       <c r="B1139" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="1140" spans="1:2">
@@ -11923,7 +11991,7 @@
         <v>9485429</v>
       </c>
       <c r="B1208" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="1209" spans="1:2">
@@ -11971,7 +12039,7 @@
         <v>9490290</v>
       </c>
       <c r="B1214" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="1215" spans="1:2">
@@ -11979,7 +12047,7 @@
         <v>9490297</v>
       </c>
       <c r="B1215" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="1216" spans="1:2">
@@ -12027,7 +12095,7 @@
         <v>9490683</v>
       </c>
       <c r="B1221" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="1222" spans="1:2">
@@ -12056,7 +12124,7 @@
         <v>9491792</v>
       </c>
       <c r="B1225" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="1226" spans="1:2">
@@ -12205,7 +12273,7 @@
         <v>9493545</v>
       </c>
       <c r="B1244" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="1245" spans="1:2">
@@ -12213,7 +12281,7 @@
         <v>9493546</v>
       </c>
       <c r="B1245" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="1246" spans="1:2">
@@ -12269,7 +12337,7 @@
         <v>9494482</v>
       </c>
       <c r="B1252" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="1253" spans="1:2">
@@ -12485,7 +12553,7 @@
         <v>9501886</v>
       </c>
       <c r="B1279" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="1280" spans="1:2">
@@ -12493,7 +12561,7 @@
         <v>9501912</v>
       </c>
       <c r="B1280" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="1281" spans="1:2">
@@ -12501,7 +12569,7 @@
         <v>9501917</v>
       </c>
       <c r="B1281" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="1282" spans="1:2">
@@ -12581,7 +12649,7 @@
         <v>9505015</v>
       </c>
       <c r="B1291" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="1292" spans="1:2">
@@ -12589,7 +12657,7 @@
         <v>9509659</v>
       </c>
       <c r="B1292" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="1293" spans="1:2">
@@ -12612,7 +12680,7 @@
         <v>9509755</v>
       </c>
       <c r="B1296" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="1297" spans="1:2">
@@ -12620,7 +12688,7 @@
         <v>9509801</v>
       </c>
       <c r="B1297" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="1298" spans="1:2">
@@ -12633,7 +12701,7 @@
         <v>9511662</v>
       </c>
       <c r="B1299" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="1300" spans="1:2">
@@ -12646,7 +12714,7 @@
         <v>9511883</v>
       </c>
       <c r="B1301" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="1302" spans="1:2">
@@ -12654,7 +12722,7 @@
         <v>9511884</v>
       </c>
       <c r="B1302" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="1303" spans="1:2">
@@ -12662,7 +12730,7 @@
         <v>9511885</v>
       </c>
       <c r="B1303" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="1304" spans="1:2">
@@ -12670,7 +12738,7 @@
         <v>9511886</v>
       </c>
       <c r="B1304" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="1305" spans="1:2">
@@ -12678,7 +12746,7 @@
         <v>9511887</v>
       </c>
       <c r="B1305" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="1306" spans="1:2">
@@ -12686,7 +12754,7 @@
         <v>9511888</v>
       </c>
       <c r="B1306" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="1307" spans="1:2">
@@ -12694,7 +12762,7 @@
         <v>9511889</v>
       </c>
       <c r="B1307" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="1308" spans="1:2">
@@ -12702,7 +12770,7 @@
         <v>9511890</v>
       </c>
       <c r="B1308" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="1309" spans="1:2">
@@ -12710,7 +12778,7 @@
         <v>9511891</v>
       </c>
       <c r="B1309" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="1310" spans="1:2">
@@ -12718,7 +12786,7 @@
         <v>9511892</v>
       </c>
       <c r="B1310" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="1311" spans="1:2">
@@ -12726,7 +12794,7 @@
         <v>9511893</v>
       </c>
       <c r="B1311" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="1312" spans="1:2">
@@ -12734,7 +12802,7 @@
         <v>9511894</v>
       </c>
       <c r="B1312" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="1313" spans="1:2">
@@ -12742,7 +12810,7 @@
         <v>9511896</v>
       </c>
       <c r="B1313" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="1314" spans="1:2">
@@ -12750,7 +12818,7 @@
         <v>9511897</v>
       </c>
       <c r="B1314" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="1315" spans="1:2">
@@ -12758,7 +12826,7 @@
         <v>9511921</v>
       </c>
       <c r="B1315" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
     </row>
     <row r="1316" spans="1:2">
@@ -12766,7 +12834,7 @@
         <v>9511922</v>
       </c>
       <c r="B1316" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="1317" spans="1:2">
@@ -12774,7 +12842,7 @@
         <v>9511924</v>
       </c>
       <c r="B1317" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="1318" spans="1:2">
@@ -12782,7 +12850,7 @@
         <v>9512004</v>
       </c>
       <c r="B1318" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
     </row>
     <row r="1319" spans="1:2">
@@ -12790,7 +12858,7 @@
         <v>9512005</v>
       </c>
       <c r="B1319" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="1320" spans="1:2">
@@ -12798,7 +12866,7 @@
         <v>9512010</v>
       </c>
       <c r="B1320" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="1321" spans="1:2">
@@ -12806,7 +12874,7 @@
         <v>9512016</v>
       </c>
       <c r="B1321" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="1322" spans="1:2">
@@ -12814,7 +12882,7 @@
         <v>9512021</v>
       </c>
       <c r="B1322" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="1323" spans="1:2">
@@ -12822,7 +12890,7 @@
         <v>9512022</v>
       </c>
       <c r="B1323" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="1324" spans="1:2">
@@ -12830,7 +12898,7 @@
         <v>9512023</v>
       </c>
       <c r="B1324" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="1325" spans="1:2">
@@ -12838,7 +12906,7 @@
         <v>9512024</v>
       </c>
       <c r="B1325" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="1326" spans="1:2">
@@ -12846,18 +12914,24 @@
         <v>9512335</v>
       </c>
       <c r="B1326" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="1327" spans="1:2">
       <c r="A1327">
         <v>9512343</v>
       </c>
+      <c r="B1327" t="s">
+        <v>914</v>
+      </c>
     </row>
     <row r="1328" spans="1:2">
       <c r="A1328">
         <v>9512349</v>
       </c>
+      <c r="B1328" t="s">
+        <v>915</v>
+      </c>
     </row>
     <row r="1329" spans="1:2">
       <c r="A1329">
@@ -12879,7 +12953,7 @@
         <v>9512396</v>
       </c>
       <c r="B1332" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="1333" spans="1:2">
@@ -12887,7 +12961,7 @@
         <v>9512455</v>
       </c>
       <c r="B1333" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="1334" spans="1:2">
@@ -12895,7 +12969,7 @@
         <v>9512466</v>
       </c>
       <c r="B1334" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="1335" spans="1:2">
@@ -12903,7 +12977,7 @@
         <v>9512481</v>
       </c>
       <c r="B1335" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
     </row>
     <row r="1336" spans="1:2">
@@ -12923,10 +12997,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:B1338">
-    <sortState ref="A10:B1338">
+    <sortState ref="A2:B1338">
       <sortCondition ref="A1:A1338"/>
     </sortState>
   </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="B149" r:id="rId1"/>
+    <hyperlink ref="B152" r:id="rId2"/>
+    <hyperlink ref="B156" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>